<commit_message>
Add GitHub Pages site, design docs and 0.2.0 acceptance evidence
Static site in site/ (home with interactive demo and live export preview,
install, guide, privacy, practice page with verified answer keys, 404),
self-hosted OFL fonts, real extension screenshots, and a manual-only Pages
workflow that verifies the site matches the build. Adds site QA, practice
page, grant preparation and download verification suites, PRODUCT.md and
DESIGN.md, the 0.2.0 acceptance record, packaged 0.2.0 build, and the
return summary and audit prompt for Astra. Nothing is deployed.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/artifacts/evidence/exports/browser.xlsx
+++ b/artifacts/evidence/exports/browser.xlsx
@@ -97,562 +97,634 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Catalog source 0</t>
+          <t>A long wrapped anchor with several lines of visible text</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>http://127.0.0.1:52478/catalog/0</t>
+          <t>http://127.0.0.1:52478/wrapped</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Catalog source 1</t>
+          <t>=SUM(1,2)</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>http://127.0.0.1:52478/catalog/1</t>
+          <t>http://127.0.0.1:52478/formula?value=(literal)</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Catalog source 2</t>
+          <t>&lt;img src=x onerror=alert(1)&gt;</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>http://127.0.0.1:52478/catalog/2</t>
+          <t>http://127.0.0.1:52478/html</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Catalog source 15</t>
+          <t>Email the research team</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>http://127.0.0.1:52478/catalog/15</t>
+          <t>mailto:research@example.org</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Catalog source 16</t>
+          <t>Call the lab</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>http://127.0.0.1:52478/catalog/16</t>
+          <t>tel:+15550123</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Catalog source 17</t>
+          <t>Open shadow source</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>http://127.0.0.1:52478/catalog/17</t>
+          <t>http://127.0.0.1:52478/shadow</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Attention in small systems</t>
+          <t>Catalog source 0</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>http://127.0.0.1:52478/papers/attention.pdf</t>
+          <t>http://127.0.0.1:52478/catalog/0</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Geometry, “frames” &amp; 雪</t>
+          <t>Catalog source 1</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>http://127.0.0.1:52478/papers/geometry.pdf?edition=2</t>
+          <t>http://127.0.0.1:52478/catalog/1</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Download PDF</t>
+          <t>Catalog source 2</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>http://127.0.0.1:52478/papers/attention.pdf</t>
+          <t>http://127.0.0.1:52478/catalog/2</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t/>
+          <t>Catalog source 15</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>http://127.0.0.1:52478/appendix</t>
+          <t>http://127.0.0.1:52478/catalog/15</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Visible label</t>
+          <t>Catalog source 16</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>http://127.0.0.1:52478/visible</t>
+          <t>http://127.0.0.1:52478/catalog/16</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Atlas notebook — field edition</t>
+          <t>Catalog source 17</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>http://127.0.0.1:52478/products/atlas</t>
+          <t>http://127.0.0.1:52478/catalog/17</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Open-sky telescope</t>
+          <t>Attention in small systems</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>https://example.org/telescope</t>
+          <t>http://127.0.0.1:52478/papers/attention.pdf</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>OBS-42</t>
+          <t>Geometry, “frames” &amp; 雪</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>http://127.0.0.1:52478/tickets/42</t>
+          <t>http://127.0.0.1:52478/papers/geometry.pdf?edition=2</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>OBS-43</t>
+          <t>Download PDF</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>http://127.0.0.1:52478/tickets/43</t>
+          <t>http://127.0.0.1:52478/papers/attention.pdf</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>A long wrapped anchor with several lines of visible text</t>
+          <t/>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>http://127.0.0.1:52478/wrapped</t>
+          <t>http://127.0.0.1:52478/appendix</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>=SUM(1,2)</t>
+          <t>Visible label</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>http://127.0.0.1:52478/formula?value=(literal)</t>
+          <t>http://127.0.0.1:52478/visible</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>&lt;img src=x onerror=alert(1)&gt;</t>
+          <t>Atlas notebook — field edition</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>http://127.0.0.1:52478/html</t>
+          <t>http://127.0.0.1:52478/products/atlas</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Email the research team</t>
+          <t>Open-sky telescope</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>mailto:research@example.org</t>
+          <t>https://example.org/telescope</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Call the lab</t>
+          <t>OBS-42</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>tel:+15550123</t>
+          <t>http://127.0.0.1:52478/tickets/42</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Open shadow source</t>
+          <t>OBS-43</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>http://127.0.0.1:52478/shadow</t>
+          <t>http://127.0.0.1:52478/tickets/43</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Loaded after the page</t>
+          <t>A long wrapped anchor with several lines of visible text</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>http://127.0.0.1:52478/dynamic</t>
+          <t>http://127.0.0.1:52478/wrapped</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Catalog source 0</t>
+          <t>=SUM(1,2)</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>http://127.0.0.1:52478/catalog/0</t>
+          <t>http://127.0.0.1:52478/formula?value=(literal)</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Catalog source 1</t>
+          <t>&lt;img src=x onerror=alert(1)&gt;</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>http://127.0.0.1:52478/catalog/1</t>
+          <t>http://127.0.0.1:52478/html</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Catalog source 2</t>
+          <t>Email the research team</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>http://127.0.0.1:52478/catalog/2</t>
+          <t>mailto:research@example.org</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Catalog source 3</t>
+          <t>Call the lab</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>http://127.0.0.1:52478/catalog/3</t>
+          <t>tel:+15550123</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>Catalog source 4</t>
+          <t>Open shadow source</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>http://127.0.0.1:52478/catalog/4</t>
+          <t>http://127.0.0.1:52478/shadow</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>Catalog source 5</t>
+          <t>Loaded after the page</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>http://127.0.0.1:52478/catalog/5</t>
+          <t>http://127.0.0.1:52478/dynamic</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>Catalog source 6</t>
+          <t>Catalog source 0</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>http://127.0.0.1:52478/catalog/6</t>
+          <t>http://127.0.0.1:52478/catalog/0</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>Catalog source 7</t>
+          <t>Catalog source 1</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>http://127.0.0.1:52478/catalog/7</t>
+          <t>http://127.0.0.1:52478/catalog/1</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>Catalog source 8</t>
+          <t>Catalog source 2</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>http://127.0.0.1:52478/catalog/8</t>
+          <t>http://127.0.0.1:52478/catalog/2</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>Catalog source 9</t>
+          <t>Catalog source 3</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>http://127.0.0.1:52478/catalog/9</t>
+          <t>http://127.0.0.1:52478/catalog/3</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>Catalog source 10</t>
+          <t>Catalog source 4</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>http://127.0.0.1:52478/catalog/10</t>
+          <t>http://127.0.0.1:52478/catalog/4</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>Catalog source 11</t>
+          <t>Catalog source 5</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>http://127.0.0.1:52478/catalog/11</t>
+          <t>http://127.0.0.1:52478/catalog/5</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>Catalog source 12</t>
+          <t>Catalog source 6</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>http://127.0.0.1:52478/catalog/12</t>
+          <t>http://127.0.0.1:52478/catalog/6</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>Catalog source 13</t>
+          <t>Catalog source 7</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>http://127.0.0.1:52478/catalog/13</t>
+          <t>http://127.0.0.1:52478/catalog/7</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>Catalog source 14</t>
+          <t>Catalog source 8</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>http://127.0.0.1:52478/catalog/14</t>
+          <t>http://127.0.0.1:52478/catalog/8</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>Catalog source 15</t>
+          <t>Catalog source 9</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>http://127.0.0.1:52478/catalog/15</t>
+          <t>http://127.0.0.1:52478/catalog/9</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>Catalog source 16</t>
+          <t>Catalog source 10</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>http://127.0.0.1:52478/catalog/16</t>
+          <t>http://127.0.0.1:52478/catalog/10</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>Catalog source 17</t>
+          <t>Catalog source 11</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>http://127.0.0.1:52478/catalog/17</t>
+          <t>http://127.0.0.1:52478/catalog/11</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>Catalog source 18</t>
+          <t>Catalog source 12</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>http://127.0.0.1:52478/catalog/18</t>
+          <t>http://127.0.0.1:52478/catalog/12</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>Catalog source 19</t>
+          <t>Catalog source 13</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>http://127.0.0.1:52478/catalog/19</t>
+          <t>http://127.0.0.1:52478/catalog/13</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>Source inside a frame</t>
+          <t>Catalog source 14</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>http://127.0.0.1:52478/frame-source</t>
+          <t>http://127.0.0.1:52478/catalog/14</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>The final source</t>
+          <t>Catalog source 15</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>http://127.0.0.1:52478/bottom</t>
+          <t>http://127.0.0.1:52478/catalog/15</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>Normal</t>
+          <t>Catalog source 16</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>http://127.0.0.1:52478/normal</t>
+          <t>http://127.0.0.1:52478/catalog/16</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>Email subject</t>
+          <t>Catalog source 17</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>mailto:?subject=Hello</t>
+          <t>http://127.0.0.1:52478/catalog/17</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
+          <t>Catalog source 18</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>http://127.0.0.1:52478/catalog/18</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>Catalog source 19</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>http://127.0.0.1:52478/catalog/19</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>Source inside a frame</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>http://127.0.0.1:52478/frame-source</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>The final source</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>http://127.0.0.1:52478/bottom</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>http://127.0.0.1:52478/normal</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>Email subject</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>mailto:?subject=Hello</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
           <t>Compose email</t>
         </is>
       </c>
-      <c r="B54" t="inlineStr">
+      <c r="B60" t="inlineStr">
         <is>
           <t>mailto:</t>
         </is>

</xml_diff>